<commit_message>
Fix sample_orders.xlsx: valid styles.xml xf entries
read_xlsx rejected the stdlib-generated workbook (Invalid xf entry in
styles.xml). Add proper numFmtId/fontId/fillId/borderId/xfId attributes,
a real font/fill/border, and a Normal cellStyle. Verified read_xlsx now
loads both sheets.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/excel-local-ingest/sample_orders.xlsx
+++ b/excel-local-ingest/sample_orders.xlsx
@@ -11,20 +11,34 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <fonts count="1">
-    <font/>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
   </fonts>
   <fills count="1">
-    <fill/>
+    <fill>
+      <patternFill patternType="none"/>
+    </fill>
   </fills>
   <borders count="1">
-    <border/>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
-    <xf/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="1">
-    <xf/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
   </cellXfs>
+  <cellStyles count="1">
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+  </cellStyles>
 </styleSheet>
 </file>
 

</xml_diff>